<commit_message>
Add .gitattributes to fix line endings
</commit_message>
<xml_diff>
--- a/selenium/Sales_Analysis_Project/data/input.xlsx
+++ b/selenium/Sales_Analysis_Project/data/input.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\python_Automation\selenium\Sales_Analysis_Project\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0252D534-7FE4-4EA5-BDF6-2D7F885AB2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="235">
   <si>
     <t>Order_ID</t>
   </si>
@@ -716,13 +722,16 @@
   </si>
   <si>
     <t>توصيل سريع</t>
+  </si>
+  <si>
+    <t>ORD-2000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -774,24 +783,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -829,7 +847,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -863,6 +881,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -897,9 +916,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1072,11 +1092,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N101"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N102"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1143,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1158,7 +1181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1199,7 +1222,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1243,7 +1266,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1284,7 +1307,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1325,7 +1348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1366,7 +1389,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1410,7 +1433,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1451,7 +1474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1495,7 +1518,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1539,7 +1562,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1580,7 +1603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1621,7 +1644,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1665,7 +1688,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1709,7 +1732,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1753,7 +1776,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1794,7 +1817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1838,7 +1861,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1882,7 +1905,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1923,7 +1946,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1967,7 +1990,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -2011,7 +2034,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -2052,7 +2075,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -2096,7 +2119,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -2140,7 +2163,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -2184,7 +2207,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -2228,7 +2251,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2269,7 +2292,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>41</v>
       </c>
@@ -2310,7 +2333,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -2354,7 +2377,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -2395,7 +2418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>44</v>
       </c>
@@ -2436,7 +2459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>45</v>
       </c>
@@ -2480,7 +2503,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>46</v>
       </c>
@@ -2521,7 +2544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -2562,7 +2585,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -2606,7 +2629,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>49</v>
       </c>
@@ -2647,7 +2670,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -2688,7 +2711,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>51</v>
       </c>
@@ -2729,7 +2752,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>52</v>
       </c>
@@ -2770,7 +2793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -2811,7 +2834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>54</v>
       </c>
@@ -2852,7 +2875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>55</v>
       </c>
@@ -2893,7 +2916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>56</v>
       </c>
@@ -2937,7 +2960,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -2981,7 +3004,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -3025,7 +3048,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>59</v>
       </c>
@@ -3066,7 +3089,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>60</v>
       </c>
@@ -3107,7 +3130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>61</v>
       </c>
@@ -3148,7 +3171,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>62</v>
       </c>
@@ -3189,7 +3212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>63</v>
       </c>
@@ -3233,7 +3256,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>64</v>
       </c>
@@ -3274,7 +3297,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>65</v>
       </c>
@@ -3318,7 +3341,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>66</v>
       </c>
@@ -3359,7 +3382,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>67</v>
       </c>
@@ -3400,7 +3423,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -3441,7 +3464,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>69</v>
       </c>
@@ -3482,7 +3505,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>70</v>
       </c>
@@ -3526,7 +3549,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>71</v>
       </c>
@@ -3564,7 +3587,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>72</v>
       </c>
@@ -3608,7 +3631,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -3649,7 +3672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>74</v>
       </c>
@@ -3693,7 +3716,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>75</v>
       </c>
@@ -3734,7 +3757,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>76</v>
       </c>
@@ -3778,7 +3801,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>77</v>
       </c>
@@ -3819,7 +3842,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>78</v>
       </c>
@@ -3860,7 +3883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>79</v>
       </c>
@@ -3904,7 +3927,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>80</v>
       </c>
@@ -3948,7 +3971,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>81</v>
       </c>
@@ -3992,7 +4015,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>82</v>
       </c>
@@ -4033,7 +4056,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -4074,7 +4097,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>84</v>
       </c>
@@ -4115,7 +4138,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>85</v>
       </c>
@@ -4153,7 +4176,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>86</v>
       </c>
@@ -4194,7 +4217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>87</v>
       </c>
@@ -4238,7 +4261,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>88</v>
       </c>
@@ -4258,7 +4281,7 @@
         <v>2</v>
       </c>
       <c r="G76">
-        <v>2535.3</v>
+        <v>2535.3000000000002</v>
       </c>
       <c r="H76">
         <v>19</v>
@@ -4282,7 +4305,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>89</v>
       </c>
@@ -4326,7 +4349,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>90</v>
       </c>
@@ -4367,7 +4390,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>91</v>
       </c>
@@ -4411,7 +4434,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>92</v>
       </c>
@@ -4455,7 +4478,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="81" spans="1:14">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>93</v>
       </c>
@@ -4496,7 +4519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:14">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>94</v>
       </c>
@@ -4540,7 +4563,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="83" spans="1:14">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>95</v>
       </c>
@@ -4584,7 +4607,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>96</v>
       </c>
@@ -4625,7 +4648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:14">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>97</v>
       </c>
@@ -4669,7 +4692,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="86" spans="1:14">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>98</v>
       </c>
@@ -4710,7 +4733,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>99</v>
       </c>
@@ -4754,7 +4777,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>100</v>
       </c>
@@ -4798,7 +4821,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>101</v>
       </c>
@@ -4839,7 +4862,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>102</v>
       </c>
@@ -4859,7 +4882,7 @@
         <v>3</v>
       </c>
       <c r="G90">
-        <v>1219.86</v>
+        <v>1219.8599999999999</v>
       </c>
       <c r="H90">
         <v>19</v>
@@ -4880,7 +4903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:14">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>103</v>
       </c>
@@ -4921,7 +4944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:14">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>104</v>
       </c>
@@ -4965,7 +4988,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>105</v>
       </c>
@@ -5006,7 +5029,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>106</v>
       </c>
@@ -5047,7 +5070,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:14">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>107</v>
       </c>
@@ -5091,7 +5114,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="96" spans="1:14">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>108</v>
       </c>
@@ -5132,7 +5155,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="97" spans="1:14">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>109</v>
       </c>
@@ -5170,7 +5193,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:14">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>110</v>
       </c>
@@ -5214,7 +5237,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="99" spans="1:14">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>111</v>
       </c>
@@ -5258,7 +5281,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="100" spans="1:14">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -5302,12 +5325,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="101" spans="1:14">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>113</v>
       </c>
-      <c r="B101" t="s">
-        <v>199</v>
+      <c r="B101" s="2">
+        <v>44990</v>
       </c>
       <c r="C101" t="s">
         <v>205</v>
@@ -5343,6 +5366,50 @@
         <v>4</v>
       </c>
       <c r="N101" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>234</v>
+      </c>
+      <c r="B102" t="s">
+        <v>199</v>
+      </c>
+      <c r="C102" t="s">
+        <v>205</v>
+      </c>
+      <c r="D102" t="s">
+        <v>208</v>
+      </c>
+      <c r="E102">
+        <v>5478</v>
+      </c>
+      <c r="F102">
+        <v>4</v>
+      </c>
+      <c r="G102">
+        <v>21882</v>
+      </c>
+      <c r="H102">
+        <v>0</v>
+      </c>
+      <c r="I102" t="s">
+        <v>213</v>
+      </c>
+      <c r="J102" t="s">
+        <v>218</v>
+      </c>
+      <c r="K102" t="s">
+        <v>226</v>
+      </c>
+      <c r="L102" t="s">
+        <v>228</v>
+      </c>
+      <c r="M102">
+        <v>4</v>
+      </c>
+      <c r="N102" t="s">
         <v>231</v>
       </c>
     </row>

</xml_diff>